<commit_message>
adding the methods to the metabolomics data
</commit_message>
<xml_diff>
--- a/output/metabolomics_with_C_numbers_curated.xlsx
+++ b/output/metabolomics_with_C_numbers_curated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pnnl-my.sharepoint.com/personal/lummy_monteiro_pnnl_gov/Documents/Documents/Lummy_personal/jupyter/Prototype/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oliv179/my_repos/PathwaySeeker/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="11_7EF9EE631379300E62355476585DCE3A87445610" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB01B963-12B8-2943-AD3F-3D3E9C73F661}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E93BD598-0F77-8C47-A469-D7765A59E5AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="423">
   <si>
     <t>metabolite</t>
   </si>
@@ -1283,13 +1283,22 @@
   </si>
   <si>
     <t>C00345</t>
+  </si>
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>HILIC Negative</t>
+  </si>
+  <si>
+    <t>C18 Positive</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1307,6 +1316,18 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1345,12 +1366,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1653,7 +1676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R325"/>
+  <dimension ref="A1:S325"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.1640625" bestFit="1" customWidth="1"/>
@@ -1664,9 +1687,10 @@
     <col min="14" max="16" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1721,8 +1745,11 @@
       <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S1" s="3" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -1777,8 +1804,11 @@
       <c r="R2" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S2" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1833,8 +1863,11 @@
       <c r="R3" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S3" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1880,8 +1913,11 @@
       <c r="R4" s="2" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S4" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -1936,8 +1972,11 @@
       <c r="R5" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S5" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -1992,8 +2031,11 @@
       <c r="R6" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S6" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -2048,8 +2090,11 @@
       <c r="R7" s="2" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S7" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -2104,8 +2149,11 @@
       <c r="R8" s="2" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S8" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -2160,8 +2208,11 @@
       <c r="R9" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S9" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>31</v>
       </c>
@@ -2216,8 +2267,11 @@
       <c r="R10" s="2" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S10" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -2272,8 +2326,11 @@
       <c r="R11" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S11" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>35</v>
       </c>
@@ -2328,8 +2385,11 @@
       <c r="R12" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S12" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -2384,8 +2444,11 @@
       <c r="R13" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S13" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>39</v>
       </c>
@@ -2440,8 +2503,11 @@
       <c r="R14" s="2" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S14" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -2488,8 +2554,11 @@
         <v>43862.542970000002</v>
       </c>
       <c r="R15" s="2"/>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S15" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>41</v>
       </c>
@@ -2544,8 +2613,11 @@
       <c r="R16" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S16" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -2600,8 +2672,11 @@
       <c r="R17" s="2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S17" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>45</v>
       </c>
@@ -2656,8 +2731,11 @@
       <c r="R18" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S18" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>47</v>
       </c>
@@ -2712,8 +2790,11 @@
       <c r="R19" s="2" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S19" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>48</v>
       </c>
@@ -2762,8 +2843,11 @@
       <c r="R20" s="2" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S20" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>49</v>
       </c>
@@ -2818,8 +2902,11 @@
       <c r="R21" s="2" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S21" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>50</v>
       </c>
@@ -2874,8 +2961,11 @@
       <c r="R22" s="2" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S22" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>51</v>
       </c>
@@ -2930,8 +3020,11 @@
       <c r="R23" s="2" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S23" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>53</v>
       </c>
@@ -2986,8 +3079,11 @@
       <c r="R24" s="2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S24" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>55</v>
       </c>
@@ -3042,8 +3138,11 @@
       <c r="R25" s="2" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S25" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>57</v>
       </c>
@@ -3098,8 +3197,11 @@
       <c r="R26" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S26" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>59</v>
       </c>
@@ -3154,8 +3256,11 @@
       <c r="R27" s="2" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S27" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>60</v>
       </c>
@@ -3210,8 +3315,11 @@
       <c r="R28" s="2" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S28" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>62</v>
       </c>
@@ -3266,8 +3374,11 @@
       <c r="R29" s="2" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S29" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>63</v>
       </c>
@@ -3322,8 +3433,11 @@
       <c r="R30" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S30" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>65</v>
       </c>
@@ -3378,8 +3492,11 @@
       <c r="R31" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S31" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>66</v>
       </c>
@@ -3434,8 +3551,11 @@
       <c r="R32" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S32" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>68</v>
       </c>
@@ -3490,8 +3610,11 @@
       <c r="R33" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S33" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>70</v>
       </c>
@@ -3546,8 +3669,11 @@
       <c r="R34" s="2" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S34" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>71</v>
       </c>
@@ -3602,8 +3728,11 @@
       <c r="R35" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S35" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>73</v>
       </c>
@@ -3658,8 +3787,11 @@
       <c r="R36" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S36" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>75</v>
       </c>
@@ -3714,8 +3846,11 @@
       <c r="R37" s="2" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S37" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>76</v>
       </c>
@@ -3770,8 +3905,11 @@
       <c r="R38" s="2" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S38" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>77</v>
       </c>
@@ -3826,8 +3964,11 @@
       <c r="R39" s="2" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S39" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>78</v>
       </c>
@@ -3882,8 +4023,11 @@
       <c r="R40" s="2" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S40" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>79</v>
       </c>
@@ -3938,8 +4082,11 @@
       <c r="R41" s="2" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S41" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>80</v>
       </c>
@@ -3994,8 +4141,11 @@
       <c r="R42" s="2" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S42" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>81</v>
       </c>
@@ -4050,8 +4200,11 @@
       <c r="R43" s="2" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S43" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>82</v>
       </c>
@@ -4106,8 +4259,11 @@
       <c r="R44" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S44" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>84</v>
       </c>
@@ -4162,8 +4318,11 @@
       <c r="R45" s="2" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S45" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>85</v>
       </c>
@@ -4216,8 +4375,11 @@
         <v>3513647</v>
       </c>
       <c r="R46" s="2"/>
-    </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S46" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>86</v>
       </c>
@@ -4272,8 +4434,11 @@
       <c r="R47" s="2" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S47" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>88</v>
       </c>
@@ -4328,8 +4493,11 @@
       <c r="R48" s="2" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S48" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>90</v>
       </c>
@@ -4384,8 +4552,11 @@
       <c r="R49" s="2" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S49" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>92</v>
       </c>
@@ -4438,8 +4609,11 @@
         <v>8564914</v>
       </c>
       <c r="R50" s="2"/>
-    </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S50" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>93</v>
       </c>
@@ -4494,8 +4668,11 @@
       <c r="R51" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S51" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>95</v>
       </c>
@@ -4548,8 +4725,11 @@
         <v>77926672</v>
       </c>
       <c r="R52" s="2"/>
-    </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S52" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>96</v>
       </c>
@@ -4604,8 +4784,11 @@
       <c r="R53" s="2" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S53" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>97</v>
       </c>
@@ -4660,8 +4843,11 @@
       <c r="R54" s="2" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S54" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>98</v>
       </c>
@@ -4716,8 +4902,11 @@
       <c r="R55" s="2" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S55" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="56" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>99</v>
       </c>
@@ -4772,8 +4961,11 @@
       <c r="R56" s="2" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S56" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="57" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>100</v>
       </c>
@@ -4828,8 +5020,11 @@
       <c r="R57" s="2" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S57" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="58" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>102</v>
       </c>
@@ -4884,8 +5079,11 @@
       <c r="R58" s="2" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S58" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="59" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>104</v>
       </c>
@@ -4940,8 +5138,11 @@
       <c r="R59" s="2" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S59" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="60" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>105</v>
       </c>
@@ -4996,8 +5197,11 @@
       <c r="R60" s="2" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S60" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>107</v>
       </c>
@@ -5052,8 +5256,11 @@
       <c r="R61" s="2" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S61" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="62" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>109</v>
       </c>
@@ -5108,8 +5315,11 @@
       <c r="R62" s="2" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S62" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="63" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>111</v>
       </c>
@@ -5164,8 +5374,11 @@
       <c r="R63" s="2" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S63" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="64" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>112</v>
       </c>
@@ -5218,8 +5431,11 @@
         <v>31904.722659999999</v>
       </c>
       <c r="R64" s="2"/>
-    </row>
-    <row r="65" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S64" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="65" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>113</v>
       </c>
@@ -5274,8 +5490,11 @@
       <c r="R65" s="2" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="66" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S65" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="66" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>115</v>
       </c>
@@ -5321,8 +5540,11 @@
       <c r="R66" s="2" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="67" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S66" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="67" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>117</v>
       </c>
@@ -5377,8 +5599,11 @@
       <c r="R67" s="2" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="68" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S67" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="68" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>118</v>
       </c>
@@ -5433,8 +5658,11 @@
       <c r="R68" s="2" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="69" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S68" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="69" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>119</v>
       </c>
@@ -5489,8 +5717,11 @@
       <c r="R69" s="2" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="70" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S69" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="70" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>120</v>
       </c>
@@ -5545,8 +5776,11 @@
       <c r="R70" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="71" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S70" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="71" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>122</v>
       </c>
@@ -5601,8 +5835,11 @@
       <c r="R71" s="2" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="72" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S71" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="72" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>123</v>
       </c>
@@ -5657,8 +5894,11 @@
       <c r="R72" s="2" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S72" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="73" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>125</v>
       </c>
@@ -5713,8 +5953,11 @@
       <c r="R73" s="2" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="74" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S73" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="74" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>126</v>
       </c>
@@ -5769,8 +6012,11 @@
       <c r="R74" s="2" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="75" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S74" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="75" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>128</v>
       </c>
@@ -5778,8 +6024,11 @@
         <v>19429.859380000002</v>
       </c>
       <c r="R75" s="2"/>
-    </row>
-    <row r="76" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S75" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="76" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>129</v>
       </c>
@@ -5832,8 +6081,11 @@
         <v>832530.375</v>
       </c>
       <c r="R76" s="2"/>
-    </row>
-    <row r="77" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S76" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="77" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>130</v>
       </c>
@@ -5888,8 +6140,11 @@
       <c r="R77" s="2" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="78" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S77" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="78" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>131</v>
       </c>
@@ -5944,8 +6199,11 @@
       <c r="R78" s="2" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="79" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S78" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="79" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>133</v>
       </c>
@@ -5982,8 +6240,11 @@
       <c r="R79" s="2" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="80" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S79" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="80" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>135</v>
       </c>
@@ -6038,8 +6299,11 @@
       <c r="R80" s="2" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="81" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S80" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="81" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>135</v>
       </c>
@@ -6094,8 +6358,11 @@
       <c r="R81" s="2" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="82" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S81" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="82" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>137</v>
       </c>
@@ -6150,8 +6417,11 @@
       <c r="R82" s="2" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="83" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S82" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="83" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>139</v>
       </c>
@@ -6206,8 +6476,11 @@
       <c r="R83" s="2" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="84" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S83" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="84" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>141</v>
       </c>
@@ -6262,8 +6535,11 @@
       <c r="R84" s="2" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="85" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S84" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="85" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>143</v>
       </c>
@@ -6318,8 +6594,11 @@
       <c r="R85" s="2" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S85" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="86" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>145</v>
       </c>
@@ -6374,8 +6653,11 @@
       <c r="R86" s="2" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="87" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S86" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="87" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>147</v>
       </c>
@@ -6385,8 +6667,11 @@
       <c r="R87" s="2" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="88" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S87" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="88" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>149</v>
       </c>
@@ -6441,8 +6726,11 @@
       <c r="R88" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="89" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S88" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="89" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>151</v>
       </c>
@@ -6497,8 +6785,11 @@
       <c r="R89" s="2" t="s">
         <v>381</v>
       </c>
-    </row>
-    <row r="90" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S89" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="90" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>152</v>
       </c>
@@ -6553,8 +6844,11 @@
       <c r="R90" s="2" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="91" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S90" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="91" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>153</v>
       </c>
@@ -6609,8 +6903,11 @@
       <c r="R91" s="2" t="s">
         <v>383</v>
       </c>
-    </row>
-    <row r="92" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S91" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="92" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>154</v>
       </c>
@@ -6665,8 +6962,11 @@
       <c r="R92" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="93" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S92" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="93" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>156</v>
       </c>
@@ -6719,8 +7019,11 @@
         <v>1854094.625</v>
       </c>
       <c r="R93" s="2"/>
-    </row>
-    <row r="94" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S93" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="94" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>157</v>
       </c>
@@ -6773,8 +7076,11 @@
         <v>52734.65625</v>
       </c>
       <c r="R94" s="2"/>
-    </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S94" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="95" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>158</v>
       </c>
@@ -6829,8 +7135,11 @@
       <c r="R95" s="2" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="96" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S95" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="96" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>159</v>
       </c>
@@ -6874,8 +7183,11 @@
         <v>35470.269529999998</v>
       </c>
       <c r="R96" s="2"/>
-    </row>
-    <row r="97" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S96" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="97" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>160</v>
       </c>
@@ -6930,8 +7242,11 @@
       <c r="R97" s="2" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="98" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S97" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="98" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>161</v>
       </c>
@@ -6968,8 +7283,11 @@
       <c r="R98" s="2" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S98" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="99" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>162</v>
       </c>
@@ -7024,8 +7342,11 @@
       <c r="R99" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="100" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S99" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="100" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>164</v>
       </c>
@@ -7078,8 +7399,11 @@
         <v>2376936.5</v>
       </c>
       <c r="R100" s="2"/>
-    </row>
-    <row r="101" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S100" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="101" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>165</v>
       </c>
@@ -7134,8 +7458,11 @@
       <c r="R101" s="2" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="102" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S101" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="102" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>167</v>
       </c>
@@ -7185,8 +7512,11 @@
         <v>697171.5</v>
       </c>
       <c r="R102" s="2"/>
-    </row>
-    <row r="103" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S102" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="103" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>168</v>
       </c>
@@ -7241,8 +7571,11 @@
       <c r="R103" s="2" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="104" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S103" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="104" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>169</v>
       </c>
@@ -7297,8 +7630,11 @@
       <c r="R104" s="2" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="105" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S104" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="105" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>171</v>
       </c>
@@ -7353,8 +7689,11 @@
       <c r="R105" s="2" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="106" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S105" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="106" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>173</v>
       </c>
@@ -7407,8 +7746,11 @@
         <v>142743.7812</v>
       </c>
       <c r="R106" s="2"/>
-    </row>
-    <row r="107" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S106" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="107" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>174</v>
       </c>
@@ -7458,8 +7800,11 @@
         <v>244896.42189999999</v>
       </c>
       <c r="R107" s="2"/>
-    </row>
-    <row r="108" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S107" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="108" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>175</v>
       </c>
@@ -7514,8 +7859,11 @@
       <c r="R108" s="2" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="109" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S108" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="109" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>176</v>
       </c>
@@ -7568,8 +7916,11 @@
         <v>42688256</v>
       </c>
       <c r="R109" s="2"/>
-    </row>
-    <row r="110" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S109" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="110" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>177</v>
       </c>
@@ -7624,8 +7975,11 @@
       <c r="R110" s="2" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="111" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S110" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="111" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>179</v>
       </c>
@@ -7680,8 +8034,11 @@
       <c r="R111" s="2" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S111" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="112" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>181</v>
       </c>
@@ -7736,8 +8093,11 @@
       <c r="R112" s="2" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="113" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S112" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="113" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>183</v>
       </c>
@@ -7792,8 +8152,11 @@
       <c r="R113" s="2" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="114" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S113" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="114" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>185</v>
       </c>
@@ -7846,8 +8209,11 @@
         <v>50109124</v>
       </c>
       <c r="R114" s="2"/>
-    </row>
-    <row r="115" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S114" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="115" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>186</v>
       </c>
@@ -7884,8 +8250,11 @@
       <c r="R115" s="2" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="116" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S115" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="116" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>187</v>
       </c>
@@ -7940,8 +8309,11 @@
       <c r="R116" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="117" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S116" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="117" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>189</v>
       </c>
@@ -7996,8 +8368,11 @@
       <c r="R117" s="2" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="118" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S117" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="118" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>191</v>
       </c>
@@ -8034,8 +8409,11 @@
       <c r="R118" s="2" t="s">
         <v>390</v>
       </c>
-    </row>
-    <row r="119" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S118" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="119" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>192</v>
       </c>
@@ -8090,8 +8468,11 @@
       <c r="R119" s="2" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="120" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S119" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="120" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>193</v>
       </c>
@@ -8102,8 +8483,11 @@
         <v>20440.814450000002</v>
       </c>
       <c r="R120" s="2"/>
-    </row>
-    <row r="121" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S120" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="121" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>194</v>
       </c>
@@ -8158,8 +8542,11 @@
       <c r="R121" s="2" t="s">
         <v>392</v>
       </c>
-    </row>
-    <row r="122" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S121" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="122" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>192</v>
       </c>
@@ -8214,8 +8601,11 @@
       <c r="R122" s="2" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="123" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S122" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="123" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>195</v>
       </c>
@@ -8270,8 +8660,11 @@
       <c r="R123" s="2" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="124" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S123" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="124" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>197</v>
       </c>
@@ -8326,8 +8719,11 @@
       <c r="R124" s="2" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="125" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S124" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="125" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>199</v>
       </c>
@@ -8382,8 +8778,11 @@
       <c r="R125" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="126" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S125" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="126" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>201</v>
       </c>
@@ -8438,8 +8837,11 @@
       <c r="R126" s="2" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="127" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S126" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="127" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>203</v>
       </c>
@@ -8494,8 +8896,11 @@
       <c r="R127" s="2" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="128" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S127" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="128" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>205</v>
       </c>
@@ -8550,8 +8955,11 @@
       <c r="R128" s="2" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="129" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S128" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="129" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>203</v>
       </c>
@@ -8606,8 +9014,11 @@
       <c r="R129" s="2" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="130" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S129" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="130" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>207</v>
       </c>
@@ -8662,8 +9073,11 @@
       <c r="R130" s="2" t="s">
         <v>393</v>
       </c>
-    </row>
-    <row r="131" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S130" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="131" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>208</v>
       </c>
@@ -8718,8 +9132,11 @@
       <c r="R131" s="2" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="132" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S131" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="132" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>208</v>
       </c>
@@ -8774,8 +9191,11 @@
       <c r="R132" s="2" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="133" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S132" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="133" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>209</v>
       </c>
@@ -8828,8 +9248,11 @@
         <v>1911146.75</v>
       </c>
       <c r="R133" s="2"/>
-    </row>
-    <row r="134" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S133" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="134" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>210</v>
       </c>
@@ -8882,8 +9305,11 @@
         <v>53843.824220000002</v>
       </c>
       <c r="R134" s="2"/>
-    </row>
-    <row r="135" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S134" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="135" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>211</v>
       </c>
@@ -8938,8 +9364,11 @@
       <c r="R135" s="2" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="136" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S135" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="136" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>213</v>
       </c>
@@ -8992,8 +9421,11 @@
         <v>235430.04689999999</v>
       </c>
       <c r="R136" s="2"/>
-    </row>
-    <row r="137" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S136" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="137" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>214</v>
       </c>
@@ -9048,8 +9480,11 @@
       <c r="R137" s="2" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="138" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S137" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="138" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>216</v>
       </c>
@@ -9102,8 +9537,11 @@
         <v>2241243.5</v>
       </c>
       <c r="R138" s="2"/>
-    </row>
-    <row r="139" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S138" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="139" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>217</v>
       </c>
@@ -9158,8 +9596,11 @@
       <c r="R139" s="2" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="140" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S139" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="140" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>218</v>
       </c>
@@ -9212,8 +9653,11 @@
         <v>4118773</v>
       </c>
       <c r="R140" s="2"/>
-    </row>
-    <row r="141" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S140" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="141" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>219</v>
       </c>
@@ -9268,8 +9712,11 @@
       <c r="R141" s="2" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="142" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S141" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="142" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>220</v>
       </c>
@@ -9324,8 +9771,11 @@
       <c r="R142" s="2" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="143" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S142" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="143" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>222</v>
       </c>
@@ -9380,8 +9830,11 @@
       <c r="R143" s="2" t="s">
         <v>397</v>
       </c>
-    </row>
-    <row r="144" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S143" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="144" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>223</v>
       </c>
@@ -9436,8 +9889,11 @@
       <c r="R144" s="2" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="145" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S144" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="145" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>225</v>
       </c>
@@ -9490,8 +9946,11 @@
         <v>681124.75</v>
       </c>
       <c r="R145" s="2"/>
-    </row>
-    <row r="146" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S145" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="146" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>226</v>
       </c>
@@ -9544,8 +10003,11 @@
         <v>45026488</v>
       </c>
       <c r="R146" s="2"/>
-    </row>
-    <row r="147" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S146" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="147" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>227</v>
       </c>
@@ -9600,8 +10062,11 @@
       <c r="R147" s="2" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="148" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S147" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="148" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>229</v>
       </c>
@@ -9654,8 +10119,11 @@
         <v>25166850</v>
       </c>
       <c r="R148" s="2"/>
-    </row>
-    <row r="149" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S148" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="149" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>230</v>
       </c>
@@ -9710,8 +10178,11 @@
       <c r="R149" s="2" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="150" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S149" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="150" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>232</v>
       </c>
@@ -9766,8 +10237,11 @@
       <c r="R150" s="2" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="151" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S150" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="151" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>234</v>
       </c>
@@ -9820,8 +10294,11 @@
         <v>9700636</v>
       </c>
       <c r="R151" s="2"/>
-    </row>
-    <row r="152" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S151" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="152" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>235</v>
       </c>
@@ -9876,8 +10353,11 @@
       <c r="R152" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="153" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S152" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="153" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>237</v>
       </c>
@@ -9930,8 +10410,11 @@
         <v>2138984.75</v>
       </c>
       <c r="R153" s="2"/>
-    </row>
-    <row r="154" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S153" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="154" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>238</v>
       </c>
@@ -9986,8 +10469,11 @@
       <c r="R154" s="2" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="155" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S154" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="155" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>239</v>
       </c>
@@ -10042,8 +10528,11 @@
       <c r="R155" s="2" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="156" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S155" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="156" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>240</v>
       </c>
@@ -10098,8 +10587,11 @@
       <c r="R156" s="2" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="157" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S156" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="157" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>241</v>
       </c>
@@ -10154,8 +10646,11 @@
       <c r="R157" s="2" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="158" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S157" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="158" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>243</v>
       </c>
@@ -10208,8 +10703,11 @@
         <v>8469816</v>
       </c>
       <c r="R158" s="2"/>
-    </row>
-    <row r="159" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S158" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="159" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>244</v>
       </c>
@@ -10264,8 +10762,11 @@
       <c r="R159" s="2" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="160" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S159" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="160" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>245</v>
       </c>
@@ -10318,8 +10819,11 @@
         <v>8469816</v>
       </c>
       <c r="R160" s="2"/>
-    </row>
-    <row r="161" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S160" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="161" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>246</v>
       </c>
@@ -10374,8 +10878,11 @@
       <c r="R161" s="2" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="162" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S161" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="162" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>248</v>
       </c>
@@ -10428,8 +10935,11 @@
         <v>1008812.5</v>
       </c>
       <c r="R162" s="2"/>
-    </row>
-    <row r="163" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S162" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="163" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>249</v>
       </c>
@@ -10484,8 +10994,11 @@
       <c r="R163" s="2" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="164" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S163" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="164" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>251</v>
       </c>
@@ -10540,8 +11053,11 @@
       <c r="R164" s="2" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="165" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S164" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="165" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>253</v>
       </c>
@@ -10596,8 +11112,11 @@
       <c r="R165" s="2" t="s">
         <v>399</v>
       </c>
-    </row>
-    <row r="166" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S165" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="166" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>254</v>
       </c>
@@ -10652,8 +11171,11 @@
       <c r="R166" s="2" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="167" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S166" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="167" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>256</v>
       </c>
@@ -10708,8 +11230,11 @@
       <c r="R167" s="2" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="168" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S167" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="168" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>258</v>
       </c>
@@ -10764,8 +11289,11 @@
       <c r="R168" s="2" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="169" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S168" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="169" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>260</v>
       </c>
@@ -10820,8 +11348,11 @@
       <c r="R169" s="2" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="170" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S169" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="170" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>261</v>
       </c>
@@ -10874,8 +11405,11 @@
         <v>6325590.5</v>
       </c>
       <c r="R170" s="2"/>
-    </row>
-    <row r="171" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S170" s="4" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="171" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>262</v>
       </c>
@@ -10930,8 +11464,11 @@
       <c r="R171" s="2" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="172" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S171" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="172" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>264</v>
       </c>
@@ -10986,8 +11523,11 @@
       <c r="R172" s="2" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="173" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S172" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="173" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>265</v>
       </c>
@@ -11036,8 +11576,11 @@
       <c r="R173" s="2" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="174" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S173" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="174" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>23</v>
       </c>
@@ -11053,16 +11596,22 @@
       <c r="R174" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="175" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S174" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="175" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>267</v>
       </c>
       <c r="R175" s="2" t="s">
         <v>401</v>
       </c>
-    </row>
-    <row r="176" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S175" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="176" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>33</v>
       </c>
@@ -11117,8 +11666,11 @@
       <c r="R176" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="177" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S176" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="177" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>37</v>
       </c>
@@ -11173,8 +11725,11 @@
       <c r="R177" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="178" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S177" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="178" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>37</v>
       </c>
@@ -11226,8 +11781,11 @@
       <c r="R178" s="2" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="179" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S178" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="179" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>269</v>
       </c>
@@ -11282,8 +11840,11 @@
       <c r="R179" s="2" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="180" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S179" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="180" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>40</v>
       </c>
@@ -11336,8 +11897,11 @@
         <v>1208290.75</v>
       </c>
       <c r="R180" s="2"/>
-    </row>
-    <row r="181" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S180" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="181" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>271</v>
       </c>
@@ -11359,8 +11923,11 @@
       <c r="R181" s="2" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="182" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S181" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="182" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>41</v>
       </c>
@@ -11370,8 +11937,11 @@
       <c r="R182" s="2" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="183" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S182" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="183" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>273</v>
       </c>
@@ -11426,8 +11996,11 @@
       <c r="R183" s="2" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="184" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S183" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="184" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>48</v>
       </c>
@@ -11482,8 +12055,11 @@
       <c r="R184" s="2" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="185" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S184" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="185" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>50</v>
       </c>
@@ -11538,8 +12114,11 @@
       <c r="R185" s="2" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="186" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S185" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="186" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>51</v>
       </c>
@@ -11594,8 +12173,11 @@
       <c r="R186" s="2" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="187" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S186" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="187" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>55</v>
       </c>
@@ -11650,8 +12232,11 @@
       <c r="R187" s="2" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="188" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S187" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="188" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>59</v>
       </c>
@@ -11706,8 +12291,11 @@
       <c r="R188" s="2" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="189" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S188" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="189" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>63</v>
       </c>
@@ -11762,8 +12350,11 @@
       <c r="R189" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="190" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S189" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="190" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>62</v>
       </c>
@@ -11818,8 +12409,11 @@
       <c r="R190" s="2" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="191" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S190" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="191" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>65</v>
       </c>
@@ -11874,8 +12468,11 @@
       <c r="R191" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="192" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S191" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="192" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>70</v>
       </c>
@@ -11930,8 +12527,11 @@
       <c r="R192" s="2" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="193" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S192" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="193" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>275</v>
       </c>
@@ -11971,8 +12571,11 @@
       <c r="R193" s="2" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="194" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S193" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="194" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>75</v>
       </c>
@@ -12021,8 +12624,11 @@
       <c r="R194" s="2" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="195" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S194" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="195" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>277</v>
       </c>
@@ -12077,8 +12683,11 @@
       <c r="R195" s="2" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="196" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S195" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="196" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>279</v>
       </c>
@@ -12133,8 +12742,11 @@
       <c r="R196" s="2" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="197" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S196" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="197" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>281</v>
       </c>
@@ -12187,8 +12799,11 @@
         <v>316658.90620000003</v>
       </c>
       <c r="R197" s="2"/>
-    </row>
-    <row r="198" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S197" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="198" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>282</v>
       </c>
@@ -12243,8 +12858,11 @@
       <c r="R198" s="2" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="199" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S198" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="199" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>283</v>
       </c>
@@ -12299,8 +12917,11 @@
       <c r="R199" s="2" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="200" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S199" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="200" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>81</v>
       </c>
@@ -12355,8 +12976,11 @@
       <c r="R200" s="2" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="201" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S200" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="201" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>285</v>
       </c>
@@ -12399,8 +13023,11 @@
       <c r="R201" s="2" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="202" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S201" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="202" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>100</v>
       </c>
@@ -12455,8 +13082,11 @@
       <c r="R202" s="2" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="203" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S202" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="203" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>99</v>
       </c>
@@ -12511,8 +13141,11 @@
       <c r="R203" s="2" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="204" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S203" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="204" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>99</v>
       </c>
@@ -12567,8 +13200,11 @@
       <c r="R204" s="2" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="205" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S204" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="205" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>287</v>
       </c>
@@ -12593,8 +13229,11 @@
       <c r="R205" s="2" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="206" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S205" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="206" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>289</v>
       </c>
@@ -12631,8 +13270,11 @@
       <c r="R206" s="2" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="207" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S206" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="207" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>102</v>
       </c>
@@ -12687,8 +13329,11 @@
       <c r="R207" s="2" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="208" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S207" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="208" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>105</v>
       </c>
@@ -12743,8 +13388,11 @@
       <c r="R208" s="2" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="209" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S208" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="209" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>109</v>
       </c>
@@ -12799,8 +13447,11 @@
       <c r="R209" s="2" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="210" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S209" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="210" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>111</v>
       </c>
@@ -12855,8 +13506,11 @@
       <c r="R210" s="2" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="211" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S210" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="211" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>111</v>
       </c>
@@ -12911,8 +13565,11 @@
       <c r="R211" s="2" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="212" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S211" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="212" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>112</v>
       </c>
@@ -12962,8 +13619,11 @@
         <v>60633.152340000001</v>
       </c>
       <c r="R212" s="2"/>
-    </row>
-    <row r="213" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S212" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="213" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>115</v>
       </c>
@@ -13018,8 +13678,11 @@
       <c r="R213" s="2" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="214" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S213" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="214" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>117</v>
       </c>
@@ -13074,8 +13737,11 @@
       <c r="R214" s="2" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="215" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S214" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="215" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>120</v>
       </c>
@@ -13130,8 +13796,11 @@
       <c r="R215" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="216" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S215" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="216" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>119</v>
       </c>
@@ -13186,8 +13855,11 @@
       <c r="R216" s="2" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="217" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S216" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="217" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>118</v>
       </c>
@@ -13242,8 +13914,11 @@
       <c r="R217" s="2" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="218" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S217" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="218" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>118</v>
       </c>
@@ -13298,8 +13973,11 @@
       <c r="R218" s="2" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="219" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S218" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="219" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>119</v>
       </c>
@@ -13354,8 +14032,11 @@
       <c r="R219" s="2" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="220" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S219" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="220" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>290</v>
       </c>
@@ -13410,8 +14091,11 @@
       <c r="R220" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="221" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S220" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="221" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>122</v>
       </c>
@@ -13466,8 +14150,11 @@
       <c r="R221" s="2" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="222" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S221" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="222" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>122</v>
       </c>
@@ -13522,8 +14209,11 @@
       <c r="R222" s="2" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="223" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S222" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="223" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>122</v>
       </c>
@@ -13578,8 +14268,11 @@
       <c r="R223" s="2" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="224" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S223" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="224" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>125</v>
       </c>
@@ -13634,8 +14327,11 @@
       <c r="R224" s="2" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="225" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S224" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="225" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>126</v>
       </c>
@@ -13690,8 +14386,11 @@
       <c r="R225" s="2" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="226" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S225" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="226" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>130</v>
       </c>
@@ -13746,8 +14445,11 @@
       <c r="R226" s="2" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="227" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S226" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="227" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>292</v>
       </c>
@@ -13802,8 +14504,11 @@
       <c r="R227" s="2" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="228" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S227" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="228" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>131</v>
       </c>
@@ -13858,8 +14563,11 @@
       <c r="R228" s="2" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="229" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S228" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="229" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>294</v>
       </c>
@@ -13914,8 +14622,11 @@
       <c r="R229" s="2" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="230" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S229" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="230" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>133</v>
       </c>
@@ -13943,8 +14654,11 @@
       <c r="R230" s="2" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="231" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S230" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="231" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>137</v>
       </c>
@@ -13999,8 +14713,11 @@
       <c r="R231" s="2" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="232" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S231" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="232" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>139</v>
       </c>
@@ -14055,8 +14772,11 @@
       <c r="R232" s="2" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="233" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S232" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="233" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>296</v>
       </c>
@@ -14111,8 +14831,11 @@
       <c r="R233" s="2" t="s">
         <v>404</v>
       </c>
-    </row>
-    <row r="234" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S233" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="234" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>143</v>
       </c>
@@ -14167,24 +14890,33 @@
       <c r="R234" s="2" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="235" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S234" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="235" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>147</v>
       </c>
       <c r="R235" s="2" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="236" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S235" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="236" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>147</v>
       </c>
       <c r="R236" s="2" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="237" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S236" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="237" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>297</v>
       </c>
@@ -14239,8 +14971,11 @@
       <c r="R237" s="2" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="238" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S237" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="238" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>149</v>
       </c>
@@ -14295,8 +15030,11 @@
       <c r="R238" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="239" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S238" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="239" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>299</v>
       </c>
@@ -14351,8 +15089,11 @@
       <c r="R239" s="2" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="240" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S239" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="240" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>151</v>
       </c>
@@ -14407,8 +15148,11 @@
       <c r="R240" s="2" t="s">
         <v>381</v>
       </c>
-    </row>
-    <row r="241" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S240" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="241" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>152</v>
       </c>
@@ -14463,8 +15207,11 @@
       <c r="R241" s="2" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="242" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S241" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="242" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>301</v>
       </c>
@@ -14519,8 +15266,11 @@
       <c r="R242" s="2" t="s">
         <v>405</v>
       </c>
-    </row>
-    <row r="243" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S242" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="243" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>154</v>
       </c>
@@ -14575,8 +15325,11 @@
       <c r="R243" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="244" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S243" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="244" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>157</v>
       </c>
@@ -14629,8 +15382,11 @@
         <v>690535.3125</v>
       </c>
       <c r="R244" s="2"/>
-    </row>
-    <row r="245" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S244" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="245" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>158</v>
       </c>
@@ -14685,8 +15441,11 @@
       <c r="R245" s="2" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="246" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S245" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="246" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>162</v>
       </c>
@@ -14741,8 +15500,11 @@
       <c r="R246" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="247" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S246" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="247" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>164</v>
       </c>
@@ -14795,8 +15557,11 @@
         <v>1001580.75</v>
       </c>
       <c r="R247" s="2"/>
-    </row>
-    <row r="248" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S247" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="248" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>302</v>
       </c>
@@ -14830,8 +15595,11 @@
       <c r="R248" s="2" t="s">
         <v>406</v>
       </c>
-    </row>
-    <row r="249" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S248" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="249" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>165</v>
       </c>
@@ -14886,8 +15654,11 @@
       <c r="R249" s="2" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="250" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S249" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="250" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>167</v>
       </c>
@@ -14940,8 +15711,11 @@
         <v>298821.03120000003</v>
       </c>
       <c r="R250" s="2"/>
-    </row>
-    <row r="251" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S250" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="251" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>303</v>
       </c>
@@ -14996,8 +15770,11 @@
       <c r="R251" s="2" t="s">
         <v>407</v>
       </c>
-    </row>
-    <row r="252" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S251" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="252" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>304</v>
       </c>
@@ -15052,8 +15829,11 @@
       <c r="R252" s="2" t="s">
         <v>305</v>
       </c>
-    </row>
-    <row r="253" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S252" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="253" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>306</v>
       </c>
@@ -15108,8 +15888,11 @@
       <c r="R253" s="2" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="254" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S253" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="254" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>169</v>
       </c>
@@ -15164,8 +15947,11 @@
       <c r="R254" s="2" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="255" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S254" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="255" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>174</v>
       </c>
@@ -15206,8 +15992,11 @@
         <v>22449.025389999999</v>
       </c>
       <c r="R255" s="2"/>
-    </row>
-    <row r="256" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S255" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="256" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>174</v>
       </c>
@@ -15248,8 +16037,11 @@
         <v>22315.646479999999</v>
       </c>
       <c r="R256" s="2"/>
-    </row>
-    <row r="257" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S256" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="257" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>175</v>
       </c>
@@ -15304,8 +16096,11 @@
       <c r="R257" s="2" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="258" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S257" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="258" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>308</v>
       </c>
@@ -15360,8 +16155,11 @@
       <c r="R258" s="2" t="s">
         <v>408</v>
       </c>
-    </row>
-    <row r="259" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S258" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="259" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>309</v>
       </c>
@@ -15414,8 +16212,11 @@
         <v>1656377</v>
       </c>
       <c r="R259" s="2"/>
-    </row>
-    <row r="260" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S259" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="260" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>310</v>
       </c>
@@ -15468,8 +16269,11 @@
         <v>395539.6875</v>
       </c>
       <c r="R260" s="2"/>
-    </row>
-    <row r="261" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S260" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="261" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
         <v>179</v>
       </c>
@@ -15524,8 +16328,11 @@
       <c r="R261" s="2" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="262" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S261" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="262" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
         <v>181</v>
       </c>
@@ -15580,8 +16387,11 @@
       <c r="R262" s="2" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="263" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S262" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="263" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
         <v>311</v>
       </c>
@@ -15636,8 +16446,11 @@
       <c r="R263" s="2" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="264" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S263" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="264" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
         <v>312</v>
       </c>
@@ -15665,16 +16478,22 @@
       <c r="R264" s="2" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="265" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S264" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="265" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
         <v>314</v>
       </c>
       <c r="R265" s="2" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="266" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S265" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="266" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
         <v>316</v>
       </c>
@@ -15729,8 +16548,11 @@
       <c r="R266" s="2" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="267" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S266" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="267" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
         <v>187</v>
       </c>
@@ -15785,8 +16607,11 @@
       <c r="R267" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="268" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S267" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="268" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
         <v>186</v>
       </c>
@@ -15841,16 +16666,22 @@
       <c r="R268" s="2" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="269" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S268" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="269" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
         <v>191</v>
       </c>
       <c r="R269" s="2" t="s">
         <v>390</v>
       </c>
-    </row>
-    <row r="270" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S269" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="270" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
         <v>318</v>
       </c>
@@ -15896,8 +16727,11 @@
       <c r="R270" s="2" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="271" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S270" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="271" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A271" t="s">
         <v>192</v>
       </c>
@@ -15952,8 +16786,11 @@
       <c r="R271" s="2" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="272" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S271" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="272" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A272" t="s">
         <v>194</v>
       </c>
@@ -16008,8 +16845,11 @@
       <c r="R272" s="2" t="s">
         <v>392</v>
       </c>
-    </row>
-    <row r="273" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S272" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="273" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
         <v>193</v>
       </c>
@@ -16023,8 +16863,11 @@
         <v>39311.121090000001</v>
       </c>
       <c r="R273" s="2"/>
-    </row>
-    <row r="274" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S273" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="274" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A274" t="s">
         <v>320</v>
       </c>
@@ -16079,8 +16922,11 @@
       <c r="R274" s="2" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="275" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S274" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="275" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A275" t="s">
         <v>197</v>
       </c>
@@ -16135,8 +16981,11 @@
       <c r="R275" s="2" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="276" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S275" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="276" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A276" t="s">
         <v>199</v>
       </c>
@@ -16191,8 +17040,11 @@
       <c r="R276" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="277" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S276" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="277" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A277" t="s">
         <v>205</v>
       </c>
@@ -16247,8 +17099,11 @@
       <c r="R277" s="2" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="278" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S277" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="278" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A278" t="s">
         <v>322</v>
       </c>
@@ -16303,8 +17158,11 @@
       <c r="R278" s="2" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="279" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S278" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="279" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A279" t="s">
         <v>208</v>
       </c>
@@ -16359,8 +17217,11 @@
       <c r="R279" s="2" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="280" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S279" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="280" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A280" t="s">
         <v>324</v>
       </c>
@@ -16415,8 +17276,11 @@
       <c r="R280" s="2" t="s">
         <v>411</v>
       </c>
-    </row>
-    <row r="281" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S280" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="281" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A281" t="s">
         <v>324</v>
       </c>
@@ -16471,8 +17335,11 @@
       <c r="R281" s="2" t="s">
         <v>411</v>
       </c>
-    </row>
-    <row r="282" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S281" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="282" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A282" t="s">
         <v>325</v>
       </c>
@@ -16527,8 +17394,11 @@
       <c r="R282" s="2" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="283" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S282" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="283" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A283" t="s">
         <v>211</v>
       </c>
@@ -16583,16 +17453,22 @@
       <c r="R283" s="2" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="284" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S283" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="284" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A284" t="s">
         <v>326</v>
       </c>
       <c r="R284" s="2" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="285" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S284" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="285" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A285" t="s">
         <v>328</v>
       </c>
@@ -16647,8 +17523,11 @@
       <c r="R285" s="2" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="286" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S285" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="286" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A286" t="s">
         <v>213</v>
       </c>
@@ -16701,8 +17580,11 @@
         <v>204697.17189999999</v>
       </c>
       <c r="R286" s="2"/>
-    </row>
-    <row r="287" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S286" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="287" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A287" t="s">
         <v>329</v>
       </c>
@@ -16757,8 +17639,11 @@
       <c r="R287" s="2" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="288" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S287" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="288" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A288" t="s">
         <v>329</v>
       </c>
@@ -16813,8 +17698,11 @@
       <c r="R288" s="2" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="289" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S288" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="289" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A289" t="s">
         <v>214</v>
       </c>
@@ -16869,8 +17757,11 @@
       <c r="R289" s="2" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="290" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S289" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="290" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A290" t="s">
         <v>216</v>
       </c>
@@ -16923,8 +17814,11 @@
         <v>516707.25</v>
       </c>
       <c r="R290" s="2"/>
-    </row>
-    <row r="291" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S290" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="291" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A291" t="s">
         <v>219</v>
       </c>
@@ -16979,8 +17873,11 @@
       <c r="R291" s="2" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="292" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S291" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="292" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A292" t="s">
         <v>219</v>
       </c>
@@ -17035,8 +17932,11 @@
       <c r="R292" s="2" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="293" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S292" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="293" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A293" t="s">
         <v>331</v>
       </c>
@@ -17091,8 +17991,11 @@
       <c r="R293" s="2" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="294" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S293" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="294" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A294" t="s">
         <v>331</v>
       </c>
@@ -17147,8 +18050,11 @@
       <c r="R294" s="2" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="295" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S294" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="295" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A295" t="s">
         <v>333</v>
       </c>
@@ -17203,8 +18109,11 @@
       <c r="R295" s="2" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="296" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S295" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="296" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A296" t="s">
         <v>222</v>
       </c>
@@ -17259,8 +18168,11 @@
       <c r="R296" s="2" t="s">
         <v>397</v>
       </c>
-    </row>
-    <row r="297" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S296" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="297" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A297" t="s">
         <v>334</v>
       </c>
@@ -17313,8 +18225,11 @@
         <v>96871.890620000006</v>
       </c>
       <c r="R297" s="2"/>
-    </row>
-    <row r="298" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S297" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="298" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A298" t="s">
         <v>223</v>
       </c>
@@ -17369,8 +18284,11 @@
       <c r="R298" s="2" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="299" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S298" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="299" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A299" t="s">
         <v>226</v>
       </c>
@@ -17423,8 +18341,11 @@
         <v>51273236</v>
       </c>
       <c r="R299" s="2"/>
-    </row>
-    <row r="300" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S299" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="300" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A300" t="s">
         <v>227</v>
       </c>
@@ -17479,8 +18400,11 @@
       <c r="R300" s="2" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="301" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S300" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="301" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A301" t="s">
         <v>229</v>
       </c>
@@ -17533,8 +18457,11 @@
         <v>15713359</v>
       </c>
       <c r="R301" s="2"/>
-    </row>
-    <row r="302" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S301" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="302" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A302" t="s">
         <v>232</v>
       </c>
@@ -17589,8 +18516,11 @@
       <c r="R302" s="2" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="303" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S302" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="303" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
         <v>230</v>
       </c>
@@ -17645,8 +18575,11 @@
       <c r="R303" s="2" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="304" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S303" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="304" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A304" t="s">
         <v>335</v>
       </c>
@@ -17701,8 +18634,11 @@
       <c r="R304" s="2" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="305" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S304" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="305" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A305" t="s">
         <v>235</v>
       </c>
@@ -17757,8 +18693,11 @@
       <c r="R305" s="2" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="306" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S305" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="306" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A306" t="s">
         <v>234</v>
       </c>
@@ -17811,8 +18750,11 @@
         <v>907998.25</v>
       </c>
       <c r="R306" s="2"/>
-    </row>
-    <row r="307" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S306" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="307" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A307" t="s">
         <v>238</v>
       </c>
@@ -17867,8 +18809,11 @@
       <c r="R307" s="2" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="308" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S307" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="308" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A308" t="s">
         <v>337</v>
       </c>
@@ -17921,8 +18866,11 @@
         <v>1303111.5</v>
       </c>
       <c r="R308" s="2"/>
-    </row>
-    <row r="309" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S308" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="309" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A309" t="s">
         <v>239</v>
       </c>
@@ -17977,8 +18925,11 @@
       <c r="R309" s="2" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="310" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S309" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="310" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A310" t="s">
         <v>244</v>
       </c>
@@ -18033,8 +18984,11 @@
       <c r="R310" s="2" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="311" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S310" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="311" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A311" t="s">
         <v>245</v>
       </c>
@@ -18087,8 +19041,11 @@
         <v>2131047.5</v>
       </c>
       <c r="R311" s="2"/>
-    </row>
-    <row r="312" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S311" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="312" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A312" t="s">
         <v>338</v>
       </c>
@@ -18141,8 +19098,11 @@
         <v>733054528</v>
       </c>
       <c r="R312" s="2"/>
-    </row>
-    <row r="313" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S312" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="313" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A313" t="s">
         <v>246</v>
       </c>
@@ -18197,8 +19157,11 @@
       <c r="R313" s="2" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="314" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S313" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="314" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A314" t="s">
         <v>339</v>
       </c>
@@ -18253,8 +19216,11 @@
       <c r="R314" s="2" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="315" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S314" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="315" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A315" t="s">
         <v>251</v>
       </c>
@@ -18309,8 +19275,11 @@
       <c r="R315" s="2" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="316" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S315" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="316" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A316" t="s">
         <v>253</v>
       </c>
@@ -18365,8 +19334,11 @@
       <c r="R316" s="2" t="s">
         <v>399</v>
       </c>
-    </row>
-    <row r="317" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S316" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="317" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A317" t="s">
         <v>341</v>
       </c>
@@ -18419,8 +19391,11 @@
         <v>11415904</v>
       </c>
       <c r="R317" s="2"/>
-    </row>
-    <row r="318" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S317" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="318" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A318" t="s">
         <v>342</v>
       </c>
@@ -18475,8 +19450,11 @@
       <c r="R318" s="2" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="319" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S318" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="319" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A319" t="s">
         <v>256</v>
       </c>
@@ -18531,8 +19509,11 @@
       <c r="R319" s="2" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="320" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S319" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="320" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A320" t="s">
         <v>343</v>
       </c>
@@ -18587,8 +19568,11 @@
       <c r="R320" s="2" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="321" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S320" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="321" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A321" t="s">
         <v>258</v>
       </c>
@@ -18643,8 +19627,11 @@
       <c r="R321" s="2" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="322" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S321" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="322" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A322" t="s">
         <v>344</v>
       </c>
@@ -18699,8 +19686,11 @@
       <c r="R322" s="2" t="s">
         <v>418</v>
       </c>
-    </row>
-    <row r="323" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S322" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="323" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A323" t="s">
         <v>345</v>
       </c>
@@ -18753,8 +19743,11 @@
         <v>179169.42189999999</v>
       </c>
       <c r="R323" s="2"/>
-    </row>
-    <row r="324" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S323" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="324" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A324" t="s">
         <v>346</v>
       </c>
@@ -18807,8 +19800,11 @@
         <v>324720</v>
       </c>
       <c r="R324" s="2"/>
-    </row>
-    <row r="325" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S324" s="4" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="325" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A325" t="s">
         <v>347</v>
       </c>
@@ -18853,6 +19849,9 @@
       </c>
       <c r="R325" s="2" t="s">
         <v>419</v>
+      </c>
+      <c r="S325" s="4" t="s">
+        <v>422</v>
       </c>
     </row>
   </sheetData>

</xml_diff>